<commit_message>
bug leakage still persists
</commit_message>
<xml_diff>
--- a/equidade_consolidada.xlsx
+++ b/equidade_consolidada.xlsx
@@ -487,19 +487,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3688</v>
+        <v>3678</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6744</v>
+        <v>0.6746</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6645</v>
+        <v>0.6647</v>
       </c>
       <c r="G2" t="n">
         <v>0.6954</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4019</v>
+        <v>0.4024</v>
       </c>
     </row>
     <row r="3">
@@ -519,16 +519,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E3" t="n">
-        <v>0.637</v>
+        <v>0.6369</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6257</v>
+        <v>0.6256</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6686</v>
+        <v>0.6685</v>
       </c>
       <c r="H3" t="n">
         <v>0.4619</v>
@@ -551,19 +551,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3688</v>
+        <v>3678</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0.671</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0.6632</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.6833</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.4467</v>
       </c>
     </row>
     <row r="5">
@@ -583,19 +583,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0.6488</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0.6364</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.678</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.4569</v>
       </c>
     </row>
     <row r="6">
@@ -615,16 +615,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2852</v>
+        <v>2843</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6501</v>
+        <v>0.6498</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6471</v>
+        <v>0.6468</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6543</v>
+        <v>0.6539</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6259</v>
+        <v>0.6264999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>0.626</v>
+        <v>0.6266</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6263</v>
+        <v>0.627</v>
       </c>
       <c r="H7" t="inlineStr"/>
     </row>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2852</v>
+        <v>2843</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6478</v>
+        <v>0.6477000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6479</v>
+        <v>0.6477000000000001</v>
       </c>
       <c r="G8" t="n">
         <v>0.6478</v>
@@ -705,16 +705,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6413</v>
+        <v>0.6419</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6468</v>
+        <v>0.6473</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6392</v>
+        <v>0.64</v>
       </c>
       <c r="H9" t="inlineStr"/>
     </row>
@@ -735,19 +735,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3662</v>
+        <v>3652</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7997</v>
+        <v>0.7999000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7988</v>
+        <v>0.799</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8007</v>
+        <v>0.8008999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2255</v>
+        <v>0.2252</v>
       </c>
     </row>
     <row r="11">
@@ -767,16 +767,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7869</v>
+        <v>0.7868000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7764</v>
+        <v>0.7763</v>
       </c>
       <c r="G11" t="n">
-        <v>0.804</v>
+        <v>0.8038999999999999</v>
       </c>
       <c r="H11" t="n">
         <v>0.2267</v>
@@ -799,19 +799,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3662</v>
+        <v>3652</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8053</v>
+        <v>0.8055</v>
       </c>
       <c r="F12" t="n">
-        <v>0.8041</v>
+        <v>0.8043</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8068</v>
+        <v>0.8071</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2142</v>
+        <v>0.2139</v>
       </c>
     </row>
     <row r="13">
@@ -831,16 +831,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8072</v>
+        <v>0.8071</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.7948</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8292</v>
+        <v>0.8290999999999999</v>
       </c>
       <c r="H13" t="n">
         <v>0.1801</v>

</xml_diff>